<commit_message>
Reentrenamiento de las redes neuronales con Early Stopping
</commit_message>
<xml_diff>
--- a/metricas_evaluacion.xlsx
+++ b/metricas_evaluacion.xlsx
@@ -943,60 +943,60 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>32.48%</t>
+          <t>45.26%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>32.48%</t>
+          <t>45.26%</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>42.16%</t>
+          <t>45.96%</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>42.16%</t>
+          <t>45.96%</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>88.73%</t>
+          <t>90.30%</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>88.73%</t>
+          <t>90.30%</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>43.33%</t>
+          <t>43.30%</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>43.33%</t>
+          <t>43.30%</t>
         </is>
       </c>
       <c r="K7" t="n">
-        <v>0.3992</v>
+        <v>0.4242</v>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>39.92%</t>
+          <t>42.42%</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>72.91%</t>
+          <t>80.39%</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>72.91%</t>
+          <t>80.39%</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
@@ -1033,60 +1033,60 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>44.53%</t>
+          <t>40.15%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>44.53%</t>
+          <t>40.15%</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>46.42%</t>
+          <t>43.71%</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>46.42%</t>
+          <t>43.71%</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>90.35%</t>
+          <t>89.61%</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>90.35%</t>
+          <t>89.61%</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>47.76%</t>
+          <t>45.27%</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>47.76%</t>
+          <t>45.27%</t>
         </is>
       </c>
       <c r="K8" t="n">
-        <v>0.4572</v>
+        <v>0.4373</v>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>45.72%</t>
+          <t>43.73%</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>79.36%</t>
+          <t>79.34%</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>79.36%</t>
+          <t>79.34%</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
@@ -1123,60 +1123,60 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>43.80%</t>
+          <t>42.70%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>43.80%</t>
+          <t>42.70%</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>47.78%</t>
+          <t>47.86%</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>47.78%</t>
+          <t>47.86%</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>90.16%</t>
+          <t>90.18%</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>90.16%</t>
+          <t>90.18%</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>52.90%</t>
+          <t>50.66%</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>52.90%</t>
+          <t>50.66%</t>
         </is>
       </c>
       <c r="K9" t="n">
-        <v>0.4668</v>
+        <v>0.4776</v>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>46.68%</t>
+          <t>47.76%</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>81.42%</t>
+          <t>81.66%</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>81.42%</t>
+          <t>81.66%</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
@@ -1213,60 +1213,60 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>21.53%</t>
+          <t>16.79%</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>21.53%</t>
+          <t>16.79%</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>14.29%</t>
+          <t>11.34%</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>14.29%</t>
+          <t>11.34%</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>85.71%</t>
+          <t>84.97%</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>85.71%</t>
+          <t>84.97%</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>3.08%</t>
+          <t>4.31%</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>3.08%</t>
+          <t>4.31%</t>
         </is>
       </c>
       <c r="K10" t="n">
-        <v>0.0506</v>
+        <v>0.0611</v>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>5.06%</t>
+          <t>6.11%</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>55.57%</t>
+          <t>57.98%</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>55.57%</t>
+          <t>57.98%</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
@@ -1303,60 +1303,60 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>90.84%</t>
+          <t>93.63%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>90.84%</t>
+          <t>93.63%</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>91.19%</t>
+          <t>93.99%</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>91.19%</t>
+          <t>93.99%</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>97.69%</t>
+          <t>98.40%</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>97.69%</t>
+          <t>98.40%</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>91.53%</t>
+          <t>93.79%</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>91.53%</t>
+          <t>93.79%</t>
         </is>
       </c>
       <c r="K11" t="n">
-        <v>0.9104</v>
+        <v>0.9376</v>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>91.04%</t>
+          <t>93.76%</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>99.21%</t>
+          <t>99.65%</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>99.21%</t>
+          <t>99.65%</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
@@ -1393,60 +1393,60 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>42.76%</t>
+          <t>41.86%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>42.76%</t>
+          <t>41.86%</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>42.44%</t>
+          <t>41.65%</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>42.44%</t>
+          <t>41.65%</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>85.52%</t>
+          <t>85.31%</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>85.52%</t>
+          <t>85.31%</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>56.24%</t>
+          <t>55.46%</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>56.24%</t>
+          <t>55.46%</t>
         </is>
       </c>
       <c r="K12" t="n">
-        <v>0.4318</v>
+        <v>0.4184</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>43.18%</t>
+          <t>41.84%</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>75.07%</t>
+          <t>73.28%</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>75.07%</t>
+          <t>73.28%</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
@@ -1483,60 +1483,60 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>50.85%</t>
+          <t>49.35%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>50.85%</t>
+          <t>49.35%</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>50.75%</t>
+          <t>49.42%</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>50.75%</t>
+          <t>49.42%</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>87.59%</t>
+          <t>87.19%</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>87.59%</t>
+          <t>87.19%</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>60.61%</t>
+          <t>66.98%</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>60.61%</t>
+          <t>66.98%</t>
         </is>
       </c>
       <c r="K13" t="n">
-        <v>0.5093</v>
+        <v>0.4993</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>50.93%</t>
+          <t>49.93%</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>77.90%</t>
+          <t>81.29%</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>77.90%</t>
+          <t>81.29%</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
@@ -1573,60 +1573,60 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>21.58%</t>
+          <t>33.17%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>21.58%</t>
+          <t>33.17%</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>20.38%</t>
+          <t>33.49%</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>20.38%</t>
+          <t>33.49%</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>80.12%</t>
+          <t>83.14%</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>80.12%</t>
+          <t>83.14%</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>7.75%</t>
+          <t>16.62%</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>7.75%</t>
+          <t>16.62%</t>
         </is>
       </c>
       <c r="K14" t="n">
-        <v>0.102</v>
+        <v>0.2085</v>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>10.20%</t>
+          <t>20.85%</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>61.77%</t>
+          <t>60.33%</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>61.77%</t>
+          <t>60.33%</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
@@ -1663,60 +1663,60 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>89.51%</t>
+          <t>92.83%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>89.51%</t>
+          <t>92.83%</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>90.10%</t>
+          <t>93.20%</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>90.10%</t>
+          <t>93.20%</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>97.36%</t>
+          <t>98.19%</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>97.36%</t>
+          <t>98.19%</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>89.61%</t>
+          <t>93.08%</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>89.61%</t>
+          <t>93.08%</t>
         </is>
       </c>
       <c r="K15" t="n">
-        <v>0.8964</v>
+        <v>0.9313</v>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>89.64%</t>
+          <t>93.13%</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>98.61%</t>
+          <t>99.47%</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>98.61%</t>
+          <t>99.47%</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
@@ -1753,60 +1753,60 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>47.15%</t>
+          <t>40.66%</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>47.15%</t>
+          <t>40.66%</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>46.75%</t>
+          <t>40.79%</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>46.75%</t>
+          <t>40.79%</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>86.65%</t>
+          <t>85.09%</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>86.65%</t>
+          <t>85.09%</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>59.65%</t>
+          <t>46.57%</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>59.65%</t>
+          <t>46.57%</t>
         </is>
       </c>
       <c r="K16" t="n">
-        <v>0.4589</v>
+        <v>0.4115</v>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>45.89%</t>
+          <t>41.15%</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>76.46%</t>
+          <t>73.82%</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>76.46%</t>
+          <t>73.82%</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
@@ -1843,60 +1843,60 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>54.35%</t>
+          <t>47.55%</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>54.35%</t>
+          <t>47.55%</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>53.86%</t>
+          <t>47.19%</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>53.86%</t>
+          <t>47.19%</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>88.44%</t>
+          <t>86.72%</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>88.44%</t>
+          <t>86.72%</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>69.08%</t>
+          <t>68.20%</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>69.08%</t>
+          <t>68.20%</t>
         </is>
       </c>
       <c r="K17" t="n">
-        <v>0.5455</v>
+        <v>0.4731</v>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>54.55%</t>
+          <t>47.31%</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>77.83%</t>
+          <t>76.93%</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>77.83%</t>
+          <t>76.93%</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
@@ -1933,60 +1933,60 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>15.88%</t>
+          <t>21.18%</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>15.88%</t>
+          <t>21.18%</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>15.09%</t>
+          <t>20.00%</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>15.09%</t>
+          <t>20.00%</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>78.77%</t>
+          <t>80.00%</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>78.77%</t>
+          <t>80.00%</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>8.59%</t>
+          <t>4.24%</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>8.59%</t>
+          <t>4.24%</t>
         </is>
       </c>
       <c r="K18" t="n">
-        <v>0.1025</v>
+        <v>0.0699</v>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>10.25%</t>
+          <t>6.99%</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>60.37%</t>
+          <t>60.54%</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>60.37%</t>
+          <t>60.54%</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">

</xml_diff>